<commit_message>
Fix formula ranges and remove unused imports
Co-authored-by: yss107 <111907417+yss107@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/a/Data Analyst Assignment Data_COMPLETED.xlsx
+++ b/a/Data Analyst Assignment Data_COMPLETED.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y137"/>
+  <dimension ref="A1:Y134"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="17.13" customWidth="1" style="25" min="3" max="3"/>
@@ -9094,7 +9094,7 @@
         </is>
       </c>
       <c r="L130" s="26">
-        <f>SUM(L2:L130)</f>
+        <f>SUM(L2:L127)</f>
         <v/>
       </c>
       <c r="M130">
@@ -9109,65 +9109,47 @@
       </c>
     </row>
     <row r="132">
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Total Orders:</t>
+        </is>
+      </c>
+      <c r="L132">
+        <f>COUNTA(J2:J127)</f>
+        <v/>
+      </c>
       <c r="M132">
         <f>TEXT(B132,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="133">
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Unpaid/Pending:</t>
+        </is>
+      </c>
+      <c r="L133">
+        <f>COUNTIF(J2:J127,"Unpaid")+COUNTIF(J2:J127,"Pending")</f>
+        <v/>
+      </c>
       <c r="M133">
         <f>TEXT(B133,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="134">
+      <c r="J134" s="26" t="inlineStr">
+        <is>
+          <t>Percentage:</t>
+        </is>
+      </c>
+      <c r="L134" s="26">
+        <f>L133/L132*100&amp;"%"</f>
+        <v/>
+      </c>
       <c r="M134">
         <f>TEXT(B134,"MMMM")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="135">
-      <c r="J135" t="inlineStr">
-        <is>
-          <t>Total Orders:</t>
-        </is>
-      </c>
-      <c r="L135">
-        <f>COUNTA(J2:J135)</f>
-        <v/>
-      </c>
-      <c r="M135">
-        <f>TEXT(B135,"MMMM")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="136">
-      <c r="J136" t="inlineStr">
-        <is>
-          <t>Unpaid/Pending:</t>
-        </is>
-      </c>
-      <c r="L136">
-        <f>COUNTIF(J2:J136,"Unpaid")+COUNTIF(J2:J136,"Pending")</f>
-        <v/>
-      </c>
-      <c r="M136">
-        <f>TEXT(B136,"MMMM")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="137">
-      <c r="J137" s="26" t="inlineStr">
-        <is>
-          <t>Percentage:</t>
-        </is>
-      </c>
-      <c r="L137" s="26">
-        <f>L136/L135*100&amp;"%"</f>
-        <v/>
-      </c>
-      <c r="M137">
-        <f>TEXT(B137,"MMMM")</f>
         <v/>
       </c>
     </row>
@@ -9342,7 +9324,7 @@
       </c>
       <c r="B5" s="21" t="inlineStr">
         <is>
-          <t>Total Revenue formula: =SUM(L2:L130) (See orders sheet for formula)</t>
+          <t>Total Revenue formula: =SUM(L2:L127) (See orders sheet for formula)</t>
         </is>
       </c>
       <c r="C5" s="21" t="n"/>
@@ -36293,19 +36275,19 @@
         </is>
       </c>
       <c r="B2">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A2,orders!$M:$M,"January")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"January")</f>
         <v/>
       </c>
       <c r="C2">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A2,orders!$M:$M,"February")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"February")</f>
         <v/>
       </c>
       <c r="D2">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A2,orders!$M:$M,"March")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"March")</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A2,orders!$M:$M,"April")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"April")</f>
         <v/>
       </c>
       <c r="F2">
@@ -36320,19 +36302,19 @@
         </is>
       </c>
       <c r="B3">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A3,orders!$M:$M,"January")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"January")</f>
         <v/>
       </c>
       <c r="C3">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A3,orders!$M:$M,"February")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"February")</f>
         <v/>
       </c>
       <c r="D3">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A3,orders!$M:$M,"March")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"March")</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A3,orders!$M:$M,"April")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"April")</f>
         <v/>
       </c>
       <c r="F3">
@@ -36347,19 +36329,19 @@
         </is>
       </c>
       <c r="B4">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A4,orders!$M:$M,"January")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"January")</f>
         <v/>
       </c>
       <c r="C4">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A4,orders!$M:$M,"February")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"February")</f>
         <v/>
       </c>
       <c r="D4">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A4,orders!$M:$M,"March")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"March")</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A4,orders!$M:$M,"April")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"April")</f>
         <v/>
       </c>
       <c r="F4">
@@ -36374,19 +36356,19 @@
         </is>
       </c>
       <c r="B5">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A5,orders!$M:$M,"January")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"January")</f>
         <v/>
       </c>
       <c r="C5">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A5,orders!$M:$M,"February")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"February")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A5,orders!$M:$M,"March")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"March")</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A5,orders!$M:$M,"April")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"April")</f>
         <v/>
       </c>
       <c r="F5">
@@ -36401,19 +36383,19 @@
         </is>
       </c>
       <c r="B6">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A6,orders!$M:$M,"January")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"January")</f>
         <v/>
       </c>
       <c r="C6">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A6,orders!$M:$M,"February")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"February")</f>
         <v/>
       </c>
       <c r="D6">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A6,orders!$M:$M,"March")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"March")</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMIFS(orders!G:$G,orders!$F:$F,$A6,orders!$M:$M,"April")</f>
+        <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"April")</f>
         <v/>
       </c>
       <c r="F6">

</xml_diff>

<commit_message>
Identify and mark duplicate rows causing formula vs pivot mismatch
Co-authored-by: yss107 <111907417+yss107@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/a/Data Analyst Assignment Data_COMPLETED.xlsx
+++ b/a/Data Analyst Assignment Data_COMPLETED.xlsx
@@ -3,9 +3,10 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="orders" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Questions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Products sold" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Analysis Notes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="orders" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Questions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Products sold" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
     <numFmt numFmtId="166" formatCode="dd-mmm-yyyy"/>
     <numFmt numFmtId="167" formatCode="M/d/yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -42,6 +43,19 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -70,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -139,7 +153,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,10 +429,255 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" style="25" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>IMPORTANT: Data Quality Issues &amp; Analysis Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>1. DUPLICATE ROWS DETECTED:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The dataset contains 2 duplicate orders:</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Order O080 (East, Office Chair): appears in rows 82 &amp; 94 of orders sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Order O100 (West, Printer): appears in rows 47 &amp; 103 of orders sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   These duplicates are marked with 'DUPLICATE' in column Z of the orders sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>2. IMPACT ON CALCULATIONS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The Excel formulas calculate ALL 126 rows including duplicates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   This affects regional totals:</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   WITH DUPLICATES (Formula-based calculation):</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - West:  ₹1,858,965.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - North: ₹1,329,260.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - South: ₹1,312,220.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - East:  ₹1,104,235.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   WITHOUT DUPLICATES (Pivot table on unique rows):</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - West:  ₹1,836,405.00 (difference: -₹22,560)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - North: ₹1,329,260.00 (no change)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - South: ₹1,312,220.00 (no change)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - East:  ₹1,089,985.00 (difference: -₹14,250)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>3. RECOMMENDATION:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   For accurate analysis, remove duplicate rows before creating pivot tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The duplicate impact totals ₹36,810 in additional Net Revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>4. WHY DIFFERENT APPROACHES GIVE DIFFERENT RESULTS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Excel formulas: Process every row individually (includes duplicates)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Pivot tables: Can be configured to handle or exclude duplicates</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Manual analysis: Should identify and handle duplicates appropriately</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>5. OTHER DATA QUALITY ISSUES:</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - 1 row with missing Salesperson Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Some Unit Price values stored as text instead of numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Order Date formatting may need standardization</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y134"/>
+  <dimension ref="A1:Z134"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="17.13" customWidth="1" style="25" min="3" max="3"/>
@@ -500,6 +762,11 @@
       <c r="W1" s="4" t="n"/>
       <c r="X1" s="4" t="n"/>
       <c r="Y1" s="4" t="n"/>
+      <c r="Z1" s="27" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
@@ -3624,6 +3891,11 @@
       <c r="W47" s="21" t="n"/>
       <c r="X47" s="21" t="n"/>
       <c r="Y47" s="21" t="n"/>
+      <c r="Z47" s="29" t="inlineStr">
+        <is>
+          <t>DUPLICATE</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
@@ -6008,6 +6280,11 @@
       <c r="W82" s="21" t="n"/>
       <c r="X82" s="21" t="n"/>
       <c r="Y82" s="21" t="n"/>
+      <c r="Z82" s="29" t="inlineStr">
+        <is>
+          <t>DUPLICATE</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
@@ -6826,6 +7103,11 @@
       <c r="W94" s="21" t="n"/>
       <c r="X94" s="21" t="n"/>
       <c r="Y94" s="21" t="n"/>
+      <c r="Z94" s="29" t="inlineStr">
+        <is>
+          <t>DUPLICATE</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
@@ -7438,6 +7720,11 @@
       <c r="W103" s="21" t="n"/>
       <c r="X103" s="21" t="n"/>
       <c r="Y103" s="21" t="n"/>
+      <c r="Z103" s="29" t="inlineStr">
+        <is>
+          <t>DUPLICATE</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
@@ -9088,12 +9375,12 @@
       </c>
     </row>
     <row r="130">
-      <c r="J130" s="26" t="inlineStr">
+      <c r="J130" s="27" t="inlineStr">
         <is>
           <t>Total Revenue:</t>
         </is>
       </c>
-      <c r="L130" s="26">
+      <c r="L130" s="27">
         <f>SUM(L2:L127)</f>
         <v/>
       </c>
@@ -9139,12 +9426,12 @@
       </c>
     </row>
     <row r="134">
-      <c r="J134" s="26" t="inlineStr">
+      <c r="J134" s="27" t="inlineStr">
         <is>
           <t>Percentage:</t>
         </is>
       </c>
-      <c r="L134" s="26">
+      <c r="L134" s="27">
         <f>L133/L132*100&amp;"%"</f>
         <v/>
       </c>
@@ -9158,7 +9445,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -9214,7 +9501,7 @@
       </c>
       <c r="B2" s="21" t="inlineStr">
         <is>
-          <t>1. Duplicate Rows: There are 2 duplicate rows in the dataset. This affects analysis by inflating counts and revenue calculations, leading to inaccurate insights about sales performance and customer behavior.
+          <t>1. Duplicate Rows: There are 2 duplicate rows in the dataset (Order O080 appears in rows 81 &amp; 93, Order O100 appears in rows 46 &amp; 102). This affects analysis by inflating counts and revenue calculations. IMPORTANT: The Excel formulas include ALL rows. For accurate pivot analysis, duplicates should be removed first. With duplicates: West=₹1,858,965, East=₹1,104,235. Without duplicates: West=₹1,836,405, East=₹1,089,985.
 2. Missing Salesperson Names: 1 order(s) have missing salesperson names. This affects performance tracking, commission calculations, and prevents accurate salesperson-level analytics.
 3. Data Type Issues: 'Unit Price' is stored as text in some cells instead of numeric type, and 'Order Date' needs to be properly formatted. This prevents proper numerical operations, sorting, and date-based filtering, potentially causing calculation errors.</t>
         </is>
@@ -9289,7 +9576,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>Pivot table created. Highest Net Revenue Region: West (₹1,858,965.00)</t>
+          <t>Pivot table created. Highest Net Revenue Region: West. NOTE: Excel formulas include duplicates (₹1,858,965.00). Pivot table excluding duplicates shows ₹1,836,405.00. The 2 duplicate rows (O080 and O100) cause a difference of ₹22,560+₹14,250=₹36,810.</t>
         </is>
       </c>
       <c r="C4" s="21" t="n"/>
@@ -36227,7 +36514,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36237,32 +36524,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="27" t="inlineStr">
         <is>
           <t>January</t>
         </is>
       </c>
-      <c r="C1" s="26" t="inlineStr">
+      <c r="C1" s="27" t="inlineStr">
         <is>
           <t>February</t>
         </is>
       </c>
-      <c r="D1" s="26" t="inlineStr">
+      <c r="D1" s="27" t="inlineStr">
         <is>
           <t>March</t>
         </is>
       </c>
-      <c r="E1" s="26" t="inlineStr">
+      <c r="E1" s="27" t="inlineStr">
         <is>
           <t>April</t>
         </is>
       </c>
-      <c r="F1" s="26" t="inlineStr">
+      <c r="F1" s="27" t="inlineStr">
         <is>
           <t>Total</t>
         </is>

</xml_diff>

<commit_message>
Add visual highlighting and detailed mismatch analysis documentation
Co-authored-by: yss107 <111907417+yss107@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/a/Data Analyst Assignment Data_COMPLETED.xlsx
+++ b/a/Data Analyst Assignment Data_COMPLETED.xlsx
@@ -58,7 +58,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +77,12 @@
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -84,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -157,6 +163,20 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -474,14 +494,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">   These duplicates are marked with 'DUPLICATE' in column Z of the orders sheet.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" s="0" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
@@ -491,7 +511,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">   The Excel formulas calculate ALL 126 rows including duplicates.</t>
         </is>
@@ -505,7 +525,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" s="0" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -543,7 +563,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" s="0" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -581,7 +601,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
+      <c r="A24" s="0" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
@@ -591,21 +611,21 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">   For accurate analysis, remove duplicate rows before creating pivot tables.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">   The duplicate impact totals ₹36,810 in additional Net Revenue.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
+      <c r="A28" s="0" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
@@ -636,7 +656,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
+      <c r="A33" s="0" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
@@ -3825,73 +3845,73 @@
       <c r="Y46" s="21" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="12" t="inlineStr">
+      <c r="A47" s="30" t="inlineStr">
         <is>
           <t>O100</t>
         </is>
       </c>
-      <c r="B47" s="6" t="n">
+      <c r="B47" s="31" t="n">
         <v>45715</v>
       </c>
-      <c r="C47" s="12" t="inlineStr">
+      <c r="C47" s="30" t="inlineStr">
         <is>
           <t>Ankit</t>
         </is>
       </c>
-      <c r="D47" s="12" t="inlineStr">
+      <c r="D47" s="30" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="E47" s="12" t="inlineStr">
+      <c r="E47" s="30" t="inlineStr">
         <is>
           <t>RAHUL NAIR</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F47" s="32" t="inlineStr">
         <is>
           <t>Printer</t>
         </is>
       </c>
-      <c r="G47" s="13" t="n">
+      <c r="G47" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="H47" s="13" t="n">
+      <c r="H47" s="33" t="n">
         <v>12000</v>
       </c>
-      <c r="I47" s="13" t="n">
+      <c r="I47" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="J47" s="12" t="inlineStr">
+      <c r="J47" s="30" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="K47" s="13">
+      <c r="K47" s="33">
         <f>IF(J47="Paid",G47*H47*(1-I47/100),"")</f>
         <v/>
       </c>
-      <c r="L47" s="13">
+      <c r="L47" s="33">
         <f>G47*H47</f>
         <v/>
       </c>
-      <c r="M47" s="13">
+      <c r="M47" s="33">
         <f>TEXT(B47,"MMMM")</f>
         <v/>
       </c>
-      <c r="N47" s="21" t="n"/>
-      <c r="O47" s="21" t="n"/>
-      <c r="P47" s="21" t="n"/>
-      <c r="Q47" s="21" t="n"/>
-      <c r="R47" s="21" t="n"/>
-      <c r="S47" s="21" t="n"/>
-      <c r="T47" s="21" t="n"/>
-      <c r="U47" s="21" t="n"/>
-      <c r="V47" s="21" t="n"/>
-      <c r="W47" s="21" t="n"/>
-      <c r="X47" s="21" t="n"/>
-      <c r="Y47" s="21" t="n"/>
-      <c r="Z47" s="29" t="inlineStr">
+      <c r="N47" s="34" t="n"/>
+      <c r="O47" s="34" t="n"/>
+      <c r="P47" s="34" t="n"/>
+      <c r="Q47" s="34" t="n"/>
+      <c r="R47" s="34" t="n"/>
+      <c r="S47" s="34" t="n"/>
+      <c r="T47" s="34" t="n"/>
+      <c r="U47" s="34" t="n"/>
+      <c r="V47" s="34" t="n"/>
+      <c r="W47" s="34" t="n"/>
+      <c r="X47" s="34" t="n"/>
+      <c r="Y47" s="34" t="n"/>
+      <c r="Z47" s="35" t="inlineStr">
         <is>
           <t>DUPLICATE</t>
         </is>
@@ -6214,73 +6234,73 @@
       <c r="Y81" s="21" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="12" t="inlineStr">
+      <c r="A82" s="30" t="inlineStr">
         <is>
           <t>O080</t>
         </is>
       </c>
-      <c r="B82" s="6" t="n">
+      <c r="B82" s="31" t="n">
         <v>45776</v>
       </c>
-      <c r="C82" s="12" t="inlineStr">
+      <c r="C82" s="30" t="inlineStr">
         <is>
           <t>Sunaina</t>
         </is>
       </c>
-      <c r="D82" s="12" t="inlineStr">
+      <c r="D82" s="30" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="E82" s="12" t="inlineStr">
+      <c r="E82" s="30" t="inlineStr">
         <is>
           <t>RIYA GUPTA</t>
         </is>
       </c>
-      <c r="F82" s="7" t="inlineStr">
+      <c r="F82" s="32" t="inlineStr">
         <is>
           <t>Office Chair</t>
         </is>
       </c>
-      <c r="G82" s="13" t="n">
+      <c r="G82" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="H82" s="13" t="n">
+      <c r="H82" s="33" t="n">
         <v>7500</v>
       </c>
-      <c r="I82" s="13" t="n">
+      <c r="I82" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="J82" s="12" t="inlineStr">
+      <c r="J82" s="30" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="K82" s="13">
+      <c r="K82" s="33">
         <f>IF(J82="Paid",G82*H82*(1-I82/100),"")</f>
         <v/>
       </c>
-      <c r="L82" s="13">
+      <c r="L82" s="33">
         <f>G82*H82</f>
         <v/>
       </c>
-      <c r="M82" s="13">
+      <c r="M82" s="33">
         <f>TEXT(B82,"MMMM")</f>
         <v/>
       </c>
-      <c r="N82" s="21" t="n"/>
-      <c r="O82" s="21" t="n"/>
-      <c r="P82" s="21" t="n"/>
-      <c r="Q82" s="21" t="n"/>
-      <c r="R82" s="21" t="n"/>
-      <c r="S82" s="21" t="n"/>
-      <c r="T82" s="21" t="n"/>
-      <c r="U82" s="21" t="n"/>
-      <c r="V82" s="21" t="n"/>
-      <c r="W82" s="21" t="n"/>
-      <c r="X82" s="21" t="n"/>
-      <c r="Y82" s="21" t="n"/>
-      <c r="Z82" s="29" t="inlineStr">
+      <c r="N82" s="34" t="n"/>
+      <c r="O82" s="34" t="n"/>
+      <c r="P82" s="34" t="n"/>
+      <c r="Q82" s="34" t="n"/>
+      <c r="R82" s="34" t="n"/>
+      <c r="S82" s="34" t="n"/>
+      <c r="T82" s="34" t="n"/>
+      <c r="U82" s="34" t="n"/>
+      <c r="V82" s="34" t="n"/>
+      <c r="W82" s="34" t="n"/>
+      <c r="X82" s="34" t="n"/>
+      <c r="Y82" s="34" t="n"/>
+      <c r="Z82" s="35" t="inlineStr">
         <is>
           <t>DUPLICATE</t>
         </is>
@@ -7037,73 +7057,73 @@
       <c r="Y93" s="21" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="12" t="inlineStr">
+      <c r="A94" s="30" t="inlineStr">
         <is>
           <t>O080</t>
         </is>
       </c>
-      <c r="B94" s="6" t="n">
+      <c r="B94" s="31" t="n">
         <v>45776</v>
       </c>
-      <c r="C94" s="12" t="inlineStr">
+      <c r="C94" s="30" t="inlineStr">
         <is>
           <t>Sunaina</t>
         </is>
       </c>
-      <c r="D94" s="12" t="inlineStr">
+      <c r="D94" s="30" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="E94" s="12" t="inlineStr">
+      <c r="E94" s="30" t="inlineStr">
         <is>
           <t>RIYA GUPTA</t>
         </is>
       </c>
-      <c r="F94" s="7" t="inlineStr">
+      <c r="F94" s="32" t="inlineStr">
         <is>
           <t>Office Chair</t>
         </is>
       </c>
-      <c r="G94" s="13" t="n">
+      <c r="G94" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="H94" s="13" t="n">
+      <c r="H94" s="33" t="n">
         <v>7500</v>
       </c>
-      <c r="I94" s="13" t="n">
+      <c r="I94" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="J94" s="12" t="inlineStr">
+      <c r="J94" s="30" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="K94" s="13">
+      <c r="K94" s="33">
         <f>IF(J94="Paid",G94*H94*(1-I94/100),"")</f>
         <v/>
       </c>
-      <c r="L94" s="13">
+      <c r="L94" s="33">
         <f>G94*H94</f>
         <v/>
       </c>
-      <c r="M94" s="13">
+      <c r="M94" s="33">
         <f>TEXT(B94,"MMMM")</f>
         <v/>
       </c>
-      <c r="N94" s="21" t="n"/>
-      <c r="O94" s="21" t="n"/>
-      <c r="P94" s="21" t="n"/>
-      <c r="Q94" s="21" t="n"/>
-      <c r="R94" s="21" t="n"/>
-      <c r="S94" s="21" t="n"/>
-      <c r="T94" s="21" t="n"/>
-      <c r="U94" s="21" t="n"/>
-      <c r="V94" s="21" t="n"/>
-      <c r="W94" s="21" t="n"/>
-      <c r="X94" s="21" t="n"/>
-      <c r="Y94" s="21" t="n"/>
-      <c r="Z94" s="29" t="inlineStr">
+      <c r="N94" s="34" t="n"/>
+      <c r="O94" s="34" t="n"/>
+      <c r="P94" s="34" t="n"/>
+      <c r="Q94" s="34" t="n"/>
+      <c r="R94" s="34" t="n"/>
+      <c r="S94" s="34" t="n"/>
+      <c r="T94" s="34" t="n"/>
+      <c r="U94" s="34" t="n"/>
+      <c r="V94" s="34" t="n"/>
+      <c r="W94" s="34" t="n"/>
+      <c r="X94" s="34" t="n"/>
+      <c r="Y94" s="34" t="n"/>
+      <c r="Z94" s="35" t="inlineStr">
         <is>
           <t>DUPLICATE</t>
         </is>
@@ -7654,73 +7674,73 @@
       <c r="Y102" s="21" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="12" t="inlineStr">
+      <c r="A103" s="30" t="inlineStr">
         <is>
           <t>O100</t>
         </is>
       </c>
-      <c r="B103" s="6" t="n">
+      <c r="B103" s="31" t="n">
         <v>45715</v>
       </c>
-      <c r="C103" s="12" t="inlineStr">
+      <c r="C103" s="30" t="inlineStr">
         <is>
           <t>Ankit</t>
         </is>
       </c>
-      <c r="D103" s="12" t="inlineStr">
+      <c r="D103" s="30" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="E103" s="12" t="inlineStr">
+      <c r="E103" s="30" t="inlineStr">
         <is>
           <t>RAHUL NAIR</t>
         </is>
       </c>
-      <c r="F103" s="7" t="inlineStr">
+      <c r="F103" s="32" t="inlineStr">
         <is>
           <t>Printer</t>
         </is>
       </c>
-      <c r="G103" s="13" t="n">
+      <c r="G103" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="H103" s="13" t="n">
+      <c r="H103" s="33" t="n">
         <v>12000</v>
       </c>
-      <c r="I103" s="13" t="n">
+      <c r="I103" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="J103" s="12" t="inlineStr">
+      <c r="J103" s="30" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="K103" s="13">
+      <c r="K103" s="33">
         <f>IF(J103="Paid",G103*H103*(1-I103/100),"")</f>
         <v/>
       </c>
-      <c r="L103" s="13">
+      <c r="L103" s="33">
         <f>G103*H103</f>
         <v/>
       </c>
-      <c r="M103" s="13">
+      <c r="M103" s="33">
         <f>TEXT(B103,"MMMM")</f>
         <v/>
       </c>
-      <c r="N103" s="21" t="n"/>
-      <c r="O103" s="21" t="n"/>
-      <c r="P103" s="21" t="n"/>
-      <c r="Q103" s="21" t="n"/>
-      <c r="R103" s="21" t="n"/>
-      <c r="S103" s="21" t="n"/>
-      <c r="T103" s="21" t="n"/>
-      <c r="U103" s="21" t="n"/>
-      <c r="V103" s="21" t="n"/>
-      <c r="W103" s="21" t="n"/>
-      <c r="X103" s="21" t="n"/>
-      <c r="Y103" s="21" t="n"/>
-      <c r="Z103" s="29" t="inlineStr">
+      <c r="N103" s="34" t="n"/>
+      <c r="O103" s="34" t="n"/>
+      <c r="P103" s="34" t="n"/>
+      <c r="Q103" s="34" t="n"/>
+      <c r="R103" s="34" t="n"/>
+      <c r="S103" s="34" t="n"/>
+      <c r="T103" s="34" t="n"/>
+      <c r="U103" s="34" t="n"/>
+      <c r="V103" s="34" t="n"/>
+      <c r="W103" s="34" t="n"/>
+      <c r="X103" s="34" t="n"/>
+      <c r="Y103" s="34" t="n"/>
+      <c r="Z103" s="35" t="inlineStr">
         <is>
           <t>DUPLICATE</t>
         </is>
@@ -9363,13 +9383,13 @@
       <c r="Y127" s="21" t="n"/>
     </row>
     <row r="128">
-      <c r="M128">
+      <c r="M128" s="0">
         <f>TEXT(B128,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="129">
-      <c r="M129">
+      <c r="M129" s="0">
         <f>TEXT(B129,"MMMM")</f>
         <v/>
       </c>
@@ -9384,43 +9404,43 @@
         <f>SUM(L2:L127)</f>
         <v/>
       </c>
-      <c r="M130">
+      <c r="M130" s="0">
         <f>TEXT(B130,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="131">
-      <c r="M131">
+      <c r="M131" s="0">
         <f>TEXT(B131,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="132">
-      <c r="J132" t="inlineStr">
+      <c r="J132" s="0" t="inlineStr">
         <is>
           <t>Total Orders:</t>
         </is>
       </c>
-      <c r="L132">
+      <c r="L132" s="0">
         <f>COUNTA(J2:J127)</f>
         <v/>
       </c>
-      <c r="M132">
+      <c r="M132" s="0">
         <f>TEXT(B132,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="133">
-      <c r="J133" t="inlineStr">
+      <c r="J133" s="0" t="inlineStr">
         <is>
           <t>Unpaid/Pending:</t>
         </is>
       </c>
-      <c r="L133">
+      <c r="L133" s="0">
         <f>COUNTIF(J2:J127,"Unpaid")+COUNTIF(J2:J127,"Pending")</f>
         <v/>
       </c>
-      <c r="M133">
+      <c r="M133" s="0">
         <f>TEXT(B133,"MMMM")</f>
         <v/>
       </c>
@@ -9435,7 +9455,7 @@
         <f>L133/L132*100&amp;"%"</f>
         <v/>
       </c>
-      <c r="M134">
+      <c r="M134" s="0">
         <f>TEXT(B134,"MMMM")</f>
         <v/>
       </c>
@@ -36556,136 +36576,136 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="B2">
+      <c r="B2" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C2">
+      <c r="C2" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D2">
+      <c r="D2" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E2">
+      <c r="E2" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F2">
+      <c r="F2" s="0">
         <f>SUM(B2:E2)</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>Laptop</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C3">
+      <c r="C3" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D3">
+      <c r="D3" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E3">
+      <c r="E3" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F3">
+      <c r="F3" s="0">
         <f>SUM(B3:E3)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B4" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C4">
+      <c r="C4" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D4">
+      <c r="D4" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E4">
+      <c r="E4" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F4">
+      <c r="F4" s="0">
         <f>SUM(B4:E4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>Office Chair</t>
         </is>
       </c>
-      <c r="B5">
+      <c r="B5" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C5">
+      <c r="C5" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D5">
+      <c r="D5" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E5">
+      <c r="E5" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F5">
+      <c r="F5" s="0">
         <f>SUM(B5:E5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>Printer</t>
         </is>
       </c>
-      <c r="B6">
+      <c r="B6" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C6">
+      <c r="C6" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D6">
+      <c r="D6" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E6">
+      <c r="E6" s="0">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="F6" s="0">
         <f>SUM(B6:E6)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fix row number consistency in duplicate detection
Co-authored-by: yss107 <111907417+yss107@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/a/Data Analyst Assignment Data_COMPLETED.xlsx
+++ b/a/Data Analyst Assignment Data_COMPLETED.xlsx
@@ -58,7 +58,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -77,12 +77,6 @@
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -90,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -163,20 +157,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -494,14 +474,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="0" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t xml:space="preserve">   These duplicates are marked with 'DUPLICATE' in column Z of the orders sheet.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="0" t="inlineStr"/>
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
@@ -511,7 +491,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="0" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t xml:space="preserve">   The Excel formulas calculate ALL 126 rows including duplicates.</t>
         </is>
@@ -525,7 +505,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="0" t="inlineStr"/>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="28" t="inlineStr">
@@ -563,7 +543,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="0" t="inlineStr"/>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="28" t="inlineStr">
@@ -601,7 +581,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="0" t="inlineStr"/>
+      <c r="A24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
@@ -611,21 +591,21 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="0" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t xml:space="preserve">   For accurate analysis, remove duplicate rows before creating pivot tables.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="0" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t xml:space="preserve">   The duplicate impact totals ₹36,810 in additional Net Revenue.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="0" t="inlineStr"/>
+      <c r="A28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
@@ -656,7 +636,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="0" t="inlineStr"/>
+      <c r="A33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
@@ -3845,73 +3825,73 @@
       <c r="Y46" s="21" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="30" t="inlineStr">
+      <c r="A47" s="12" t="inlineStr">
         <is>
           <t>O100</t>
         </is>
       </c>
-      <c r="B47" s="31" t="n">
+      <c r="B47" s="6" t="n">
         <v>45715</v>
       </c>
-      <c r="C47" s="30" t="inlineStr">
+      <c r="C47" s="12" t="inlineStr">
         <is>
           <t>Ankit</t>
         </is>
       </c>
-      <c r="D47" s="30" t="inlineStr">
+      <c r="D47" s="12" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="E47" s="30" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>RAHUL NAIR</t>
         </is>
       </c>
-      <c r="F47" s="32" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>Printer</t>
         </is>
       </c>
-      <c r="G47" s="33" t="n">
+      <c r="G47" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H47" s="33" t="n">
+      <c r="H47" s="13" t="n">
         <v>12000</v>
       </c>
-      <c r="I47" s="33" t="n">
+      <c r="I47" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="J47" s="30" t="inlineStr">
+      <c r="J47" s="12" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="K47" s="33">
+      <c r="K47" s="13">
         <f>IF(J47="Paid",G47*H47*(1-I47/100),"")</f>
         <v/>
       </c>
-      <c r="L47" s="33">
+      <c r="L47" s="13">
         <f>G47*H47</f>
         <v/>
       </c>
-      <c r="M47" s="33">
+      <c r="M47" s="13">
         <f>TEXT(B47,"MMMM")</f>
         <v/>
       </c>
-      <c r="N47" s="34" t="n"/>
-      <c r="O47" s="34" t="n"/>
-      <c r="P47" s="34" t="n"/>
-      <c r="Q47" s="34" t="n"/>
-      <c r="R47" s="34" t="n"/>
-      <c r="S47" s="34" t="n"/>
-      <c r="T47" s="34" t="n"/>
-      <c r="U47" s="34" t="n"/>
-      <c r="V47" s="34" t="n"/>
-      <c r="W47" s="34" t="n"/>
-      <c r="X47" s="34" t="n"/>
-      <c r="Y47" s="34" t="n"/>
-      <c r="Z47" s="35" t="inlineStr">
+      <c r="N47" s="21" t="n"/>
+      <c r="O47" s="21" t="n"/>
+      <c r="P47" s="21" t="n"/>
+      <c r="Q47" s="21" t="n"/>
+      <c r="R47" s="21" t="n"/>
+      <c r="S47" s="21" t="n"/>
+      <c r="T47" s="21" t="n"/>
+      <c r="U47" s="21" t="n"/>
+      <c r="V47" s="21" t="n"/>
+      <c r="W47" s="21" t="n"/>
+      <c r="X47" s="21" t="n"/>
+      <c r="Y47" s="21" t="n"/>
+      <c r="Z47" s="29" t="inlineStr">
         <is>
           <t>DUPLICATE</t>
         </is>
@@ -6234,73 +6214,73 @@
       <c r="Y81" s="21" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="30" t="inlineStr">
+      <c r="A82" s="12" t="inlineStr">
         <is>
           <t>O080</t>
         </is>
       </c>
-      <c r="B82" s="31" t="n">
+      <c r="B82" s="6" t="n">
         <v>45776</v>
       </c>
-      <c r="C82" s="30" t="inlineStr">
+      <c r="C82" s="12" t="inlineStr">
         <is>
           <t>Sunaina</t>
         </is>
       </c>
-      <c r="D82" s="30" t="inlineStr">
+      <c r="D82" s="12" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="E82" s="30" t="inlineStr">
+      <c r="E82" s="12" t="inlineStr">
         <is>
           <t>RIYA GUPTA</t>
         </is>
       </c>
-      <c r="F82" s="32" t="inlineStr">
+      <c r="F82" s="7" t="inlineStr">
         <is>
           <t>Office Chair</t>
         </is>
       </c>
-      <c r="G82" s="33" t="n">
+      <c r="G82" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H82" s="33" t="n">
+      <c r="H82" s="13" t="n">
         <v>7500</v>
       </c>
-      <c r="I82" s="33" t="n">
+      <c r="I82" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="J82" s="30" t="inlineStr">
+      <c r="J82" s="12" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="K82" s="33">
+      <c r="K82" s="13">
         <f>IF(J82="Paid",G82*H82*(1-I82/100),"")</f>
         <v/>
       </c>
-      <c r="L82" s="33">
+      <c r="L82" s="13">
         <f>G82*H82</f>
         <v/>
       </c>
-      <c r="M82" s="33">
+      <c r="M82" s="13">
         <f>TEXT(B82,"MMMM")</f>
         <v/>
       </c>
-      <c r="N82" s="34" t="n"/>
-      <c r="O82" s="34" t="n"/>
-      <c r="P82" s="34" t="n"/>
-      <c r="Q82" s="34" t="n"/>
-      <c r="R82" s="34" t="n"/>
-      <c r="S82" s="34" t="n"/>
-      <c r="T82" s="34" t="n"/>
-      <c r="U82" s="34" t="n"/>
-      <c r="V82" s="34" t="n"/>
-      <c r="W82" s="34" t="n"/>
-      <c r="X82" s="34" t="n"/>
-      <c r="Y82" s="34" t="n"/>
-      <c r="Z82" s="35" t="inlineStr">
+      <c r="N82" s="21" t="n"/>
+      <c r="O82" s="21" t="n"/>
+      <c r="P82" s="21" t="n"/>
+      <c r="Q82" s="21" t="n"/>
+      <c r="R82" s="21" t="n"/>
+      <c r="S82" s="21" t="n"/>
+      <c r="T82" s="21" t="n"/>
+      <c r="U82" s="21" t="n"/>
+      <c r="V82" s="21" t="n"/>
+      <c r="W82" s="21" t="n"/>
+      <c r="X82" s="21" t="n"/>
+      <c r="Y82" s="21" t="n"/>
+      <c r="Z82" s="29" t="inlineStr">
         <is>
           <t>DUPLICATE</t>
         </is>
@@ -7057,73 +7037,73 @@
       <c r="Y93" s="21" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="30" t="inlineStr">
+      <c r="A94" s="12" t="inlineStr">
         <is>
           <t>O080</t>
         </is>
       </c>
-      <c r="B94" s="31" t="n">
+      <c r="B94" s="6" t="n">
         <v>45776</v>
       </c>
-      <c r="C94" s="30" t="inlineStr">
+      <c r="C94" s="12" t="inlineStr">
         <is>
           <t>Sunaina</t>
         </is>
       </c>
-      <c r="D94" s="30" t="inlineStr">
+      <c r="D94" s="12" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="E94" s="30" t="inlineStr">
+      <c r="E94" s="12" t="inlineStr">
         <is>
           <t>RIYA GUPTA</t>
         </is>
       </c>
-      <c r="F94" s="32" t="inlineStr">
+      <c r="F94" s="7" t="inlineStr">
         <is>
           <t>Office Chair</t>
         </is>
       </c>
-      <c r="G94" s="33" t="n">
+      <c r="G94" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H94" s="33" t="n">
+      <c r="H94" s="13" t="n">
         <v>7500</v>
       </c>
-      <c r="I94" s="33" t="n">
+      <c r="I94" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="J94" s="30" t="inlineStr">
+      <c r="J94" s="12" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="K94" s="33">
+      <c r="K94" s="13">
         <f>IF(J94="Paid",G94*H94*(1-I94/100),"")</f>
         <v/>
       </c>
-      <c r="L94" s="33">
+      <c r="L94" s="13">
         <f>G94*H94</f>
         <v/>
       </c>
-      <c r="M94" s="33">
+      <c r="M94" s="13">
         <f>TEXT(B94,"MMMM")</f>
         <v/>
       </c>
-      <c r="N94" s="34" t="n"/>
-      <c r="O94" s="34" t="n"/>
-      <c r="P94" s="34" t="n"/>
-      <c r="Q94" s="34" t="n"/>
-      <c r="R94" s="34" t="n"/>
-      <c r="S94" s="34" t="n"/>
-      <c r="T94" s="34" t="n"/>
-      <c r="U94" s="34" t="n"/>
-      <c r="V94" s="34" t="n"/>
-      <c r="W94" s="34" t="n"/>
-      <c r="X94" s="34" t="n"/>
-      <c r="Y94" s="34" t="n"/>
-      <c r="Z94" s="35" t="inlineStr">
+      <c r="N94" s="21" t="n"/>
+      <c r="O94" s="21" t="n"/>
+      <c r="P94" s="21" t="n"/>
+      <c r="Q94" s="21" t="n"/>
+      <c r="R94" s="21" t="n"/>
+      <c r="S94" s="21" t="n"/>
+      <c r="T94" s="21" t="n"/>
+      <c r="U94" s="21" t="n"/>
+      <c r="V94" s="21" t="n"/>
+      <c r="W94" s="21" t="n"/>
+      <c r="X94" s="21" t="n"/>
+      <c r="Y94" s="21" t="n"/>
+      <c r="Z94" s="29" t="inlineStr">
         <is>
           <t>DUPLICATE</t>
         </is>
@@ -7674,73 +7654,73 @@
       <c r="Y102" s="21" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="30" t="inlineStr">
+      <c r="A103" s="12" t="inlineStr">
         <is>
           <t>O100</t>
         </is>
       </c>
-      <c r="B103" s="31" t="n">
+      <c r="B103" s="6" t="n">
         <v>45715</v>
       </c>
-      <c r="C103" s="30" t="inlineStr">
+      <c r="C103" s="12" t="inlineStr">
         <is>
           <t>Ankit</t>
         </is>
       </c>
-      <c r="D103" s="30" t="inlineStr">
+      <c r="D103" s="12" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="E103" s="30" t="inlineStr">
+      <c r="E103" s="12" t="inlineStr">
         <is>
           <t>RAHUL NAIR</t>
         </is>
       </c>
-      <c r="F103" s="32" t="inlineStr">
+      <c r="F103" s="7" t="inlineStr">
         <is>
           <t>Printer</t>
         </is>
       </c>
-      <c r="G103" s="33" t="n">
+      <c r="G103" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H103" s="33" t="n">
+      <c r="H103" s="13" t="n">
         <v>12000</v>
       </c>
-      <c r="I103" s="33" t="n">
+      <c r="I103" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="J103" s="30" t="inlineStr">
+      <c r="J103" s="12" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="K103" s="33">
+      <c r="K103" s="13">
         <f>IF(J103="Paid",G103*H103*(1-I103/100),"")</f>
         <v/>
       </c>
-      <c r="L103" s="33">
+      <c r="L103" s="13">
         <f>G103*H103</f>
         <v/>
       </c>
-      <c r="M103" s="33">
+      <c r="M103" s="13">
         <f>TEXT(B103,"MMMM")</f>
         <v/>
       </c>
-      <c r="N103" s="34" t="n"/>
-      <c r="O103" s="34" t="n"/>
-      <c r="P103" s="34" t="n"/>
-      <c r="Q103" s="34" t="n"/>
-      <c r="R103" s="34" t="n"/>
-      <c r="S103" s="34" t="n"/>
-      <c r="T103" s="34" t="n"/>
-      <c r="U103" s="34" t="n"/>
-      <c r="V103" s="34" t="n"/>
-      <c r="W103" s="34" t="n"/>
-      <c r="X103" s="34" t="n"/>
-      <c r="Y103" s="34" t="n"/>
-      <c r="Z103" s="35" t="inlineStr">
+      <c r="N103" s="21" t="n"/>
+      <c r="O103" s="21" t="n"/>
+      <c r="P103" s="21" t="n"/>
+      <c r="Q103" s="21" t="n"/>
+      <c r="R103" s="21" t="n"/>
+      <c r="S103" s="21" t="n"/>
+      <c r="T103" s="21" t="n"/>
+      <c r="U103" s="21" t="n"/>
+      <c r="V103" s="21" t="n"/>
+      <c r="W103" s="21" t="n"/>
+      <c r="X103" s="21" t="n"/>
+      <c r="Y103" s="21" t="n"/>
+      <c r="Z103" s="29" t="inlineStr">
         <is>
           <t>DUPLICATE</t>
         </is>
@@ -9383,13 +9363,13 @@
       <c r="Y127" s="21" t="n"/>
     </row>
     <row r="128">
-      <c r="M128" s="0">
+      <c r="M128">
         <f>TEXT(B128,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="129">
-      <c r="M129" s="0">
+      <c r="M129">
         <f>TEXT(B129,"MMMM")</f>
         <v/>
       </c>
@@ -9404,43 +9384,43 @@
         <f>SUM(L2:L127)</f>
         <v/>
       </c>
-      <c r="M130" s="0">
+      <c r="M130">
         <f>TEXT(B130,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="131">
-      <c r="M131" s="0">
+      <c r="M131">
         <f>TEXT(B131,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="132">
-      <c r="J132" s="0" t="inlineStr">
+      <c r="J132" t="inlineStr">
         <is>
           <t>Total Orders:</t>
         </is>
       </c>
-      <c r="L132" s="0">
+      <c r="L132">
         <f>COUNTA(J2:J127)</f>
         <v/>
       </c>
-      <c r="M132" s="0">
+      <c r="M132">
         <f>TEXT(B132,"MMMM")</f>
         <v/>
       </c>
     </row>
     <row r="133">
-      <c r="J133" s="0" t="inlineStr">
+      <c r="J133" t="inlineStr">
         <is>
           <t>Unpaid/Pending:</t>
         </is>
       </c>
-      <c r="L133" s="0">
+      <c r="L133">
         <f>COUNTIF(J2:J127,"Unpaid")+COUNTIF(J2:J127,"Pending")</f>
         <v/>
       </c>
-      <c r="M133" s="0">
+      <c r="M133">
         <f>TEXT(B133,"MMMM")</f>
         <v/>
       </c>
@@ -9455,7 +9435,7 @@
         <f>L133/L132*100&amp;"%"</f>
         <v/>
       </c>
-      <c r="M134" s="0">
+      <c r="M134">
         <f>TEXT(B134,"MMMM")</f>
         <v/>
       </c>
@@ -9521,7 +9501,7 @@
       </c>
       <c r="B2" s="21" t="inlineStr">
         <is>
-          <t>1. Duplicate Rows: There are 2 duplicate rows in the dataset (Order O080 appears in rows 81 &amp; 93, Order O100 appears in rows 46 &amp; 102). This affects analysis by inflating counts and revenue calculations. IMPORTANT: The Excel formulas include ALL rows. For accurate pivot analysis, duplicates should be removed first. With duplicates: West=₹1,858,965, East=₹1,104,235. Without duplicates: West=₹1,836,405, East=₹1,089,985.
+          <t>1. Duplicate Rows: There are 2 duplicate rows in the dataset (Order O080 appears in rows 82 &amp; 94, Order O100 appears in rows 47 &amp; 103). This affects analysis by inflating counts and revenue calculations. IMPORTANT: The Excel formulas include ALL rows. For accurate pivot analysis, duplicates should be removed first. With duplicates: West=₹1,858,965, East=₹1,104,235. Without duplicates: West=₹1,836,405, East=₹1,089,985.
 2. Missing Salesperson Names: 1 order(s) have missing salesperson names. This affects performance tracking, commission calculations, and prevents accurate salesperson-level analytics.
 3. Data Type Issues: 'Unit Price' is stored as text in some cells instead of numeric type, and 'Order Date' needs to be properly formatted. This prevents proper numerical operations, sorting, and date-based filtering, potentially causing calculation errors.</t>
         </is>
@@ -36576,136 +36556,136 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="B2" s="0">
+      <c r="B2">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C2" s="0">
+      <c r="C2">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D2" s="0">
+      <c r="D2">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E2" s="0">
+      <c r="E2">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A2,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F2" s="0">
+      <c r="F2">
         <f>SUM(B2:E2)</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Laptop</t>
         </is>
       </c>
-      <c r="B3" s="0">
+      <c r="B3">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C3" s="0">
+      <c r="C3">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D3" s="0">
+      <c r="D3">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E3" s="0">
+      <c r="E3">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A3,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F3" s="0">
+      <c r="F3">
         <f>SUM(B3:E3)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="0" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="B4" s="0">
+      <c r="B4">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C4" s="0">
+      <c r="C4">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D4" s="0">
+      <c r="D4">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E4" s="0">
+      <c r="E4">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A4,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F4" s="0">
+      <c r="F4">
         <f>SUM(B4:E4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="0" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Office Chair</t>
         </is>
       </c>
-      <c r="B5" s="0">
+      <c r="B5">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C5" s="0">
+      <c r="C5">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D5" s="0">
+      <c r="D5">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E5" s="0">
+      <c r="E5">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A5,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F5" s="0">
+      <c r="F5">
         <f>SUM(B5:E5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="0" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Printer</t>
         </is>
       </c>
-      <c r="B6" s="0">
+      <c r="B6">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"January")</f>
         <v/>
       </c>
-      <c r="C6" s="0">
+      <c r="C6">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"February")</f>
         <v/>
       </c>
-      <c r="D6" s="0">
+      <c r="D6">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"March")</f>
         <v/>
       </c>
-      <c r="E6" s="0">
+      <c r="E6">
         <f>SUMIFS(orders!$G:$G,orders!$F:$F,$A6,orders!$M:$M,"April")</f>
         <v/>
       </c>
-      <c r="F6" s="0">
+      <c r="F6">
         <f>SUM(B6:E6)</f>
         <v/>
       </c>

</xml_diff>